<commit_message>
revisions to plot layout
</commit_message>
<xml_diff>
--- a/sccj-faculty-salary-data.xlsx
+++ b/sccj-faculty-salary-data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jyoung20/Github/sccj-faculty-salary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E1C928-6E9A-974A-A027-BE82DD0C6D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52548FA0-26DB-F045-BBB7-8815AD7E3D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="21720" xr2:uid="{390A8155-8037-4544-B779-6A79251AF3D7}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="115">
   <si>
     <t>ID</t>
   </si>
@@ -377,6 +377,9 @@
   </si>
   <si>
     <t>admin_appointment</t>
+  </si>
+  <si>
+    <t>regents</t>
   </si>
 </sst>
 </file>
@@ -736,14 +739,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718F963D-5933-5B4F-9721-1D63B7B62310}">
-  <dimension ref="A1:J224"/>
+  <dimension ref="A1:K224"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -774,8 +778,11 @@
       <c r="J1" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>109</v>
       </c>
@@ -806,8 +813,11 @@
       <c r="J2" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>75</v>
       </c>
@@ -838,8 +848,11 @@
       <c r="J3" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>76</v>
       </c>
@@ -870,8 +883,11 @@
       <c r="J4" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>77</v>
       </c>
@@ -902,8 +918,11 @@
       <c r="J5" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>78</v>
       </c>
@@ -934,8 +953,11 @@
       <c r="J6" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>79</v>
       </c>
@@ -966,8 +988,11 @@
       <c r="J7" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>80</v>
       </c>
@@ -998,8 +1023,11 @@
       <c r="J8" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>81</v>
       </c>
@@ -1030,8 +1058,11 @@
       <c r="J9" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>82</v>
       </c>
@@ -1062,8 +1093,11 @@
       <c r="J10" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>83</v>
       </c>
@@ -1094,8 +1128,11 @@
       <c r="J11" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>84</v>
       </c>
@@ -1126,8 +1163,11 @@
       <c r="J12" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>85</v>
       </c>
@@ -1158,8 +1198,11 @@
       <c r="J13" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>86</v>
       </c>
@@ -1190,8 +1233,11 @@
       <c r="J14" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>87</v>
       </c>
@@ -1222,8 +1268,11 @@
       <c r="J15" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>88</v>
       </c>
@@ -1254,8 +1303,11 @@
       <c r="J16" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1286,8 +1338,11 @@
       <c r="J17" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>91</v>
       </c>
@@ -1318,8 +1373,11 @@
       <c r="J18" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>92</v>
       </c>
@@ -1350,8 +1408,11 @@
       <c r="J19" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>93</v>
       </c>
@@ -1382,8 +1443,11 @@
       <c r="J20" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>94</v>
       </c>
@@ -1414,8 +1478,11 @@
       <c r="J21" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>95</v>
       </c>
@@ -1446,8 +1513,11 @@
       <c r="J22" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>96</v>
       </c>
@@ -1478,8 +1548,11 @@
       <c r="J23" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>97</v>
       </c>
@@ -1510,8 +1583,11 @@
       <c r="J24" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>98</v>
       </c>
@@ -1542,8 +1618,11 @@
       <c r="J25" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>99</v>
       </c>
@@ -1574,8 +1653,11 @@
       <c r="J26" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>100</v>
       </c>
@@ -1606,8 +1688,11 @@
       <c r="J27" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>101</v>
       </c>
@@ -1638,8 +1723,11 @@
       <c r="J28" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>102</v>
       </c>
@@ -1670,8 +1758,11 @@
       <c r="J29" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>103</v>
       </c>
@@ -1702,8 +1793,11 @@
       <c r="J30" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>104</v>
       </c>
@@ -1734,8 +1828,11 @@
       <c r="J31" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>105</v>
       </c>
@@ -1766,8 +1863,11 @@
       <c r="J32" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>106</v>
       </c>
@@ -1798,8 +1898,11 @@
       <c r="J33" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>75</v>
       </c>
@@ -1830,8 +1933,11 @@
       <c r="J34" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>76</v>
       </c>
@@ -1862,8 +1968,11 @@
       <c r="J35" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -1894,8 +2003,11 @@
       <c r="J36" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>78</v>
       </c>
@@ -1926,8 +2038,11 @@
       <c r="J37" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>79</v>
       </c>
@@ -1958,8 +2073,11 @@
       <c r="J38" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>80</v>
       </c>
@@ -1990,8 +2108,11 @@
       <c r="J39" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>81</v>
       </c>
@@ -2022,8 +2143,11 @@
       <c r="J40" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>82</v>
       </c>
@@ -2054,8 +2178,11 @@
       <c r="J41" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>83</v>
       </c>
@@ -2086,8 +2213,11 @@
       <c r="J42" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>84</v>
       </c>
@@ -2118,8 +2248,11 @@
       <c r="J43" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>85</v>
       </c>
@@ -2150,8 +2283,11 @@
       <c r="J44" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>86</v>
       </c>
@@ -2182,8 +2318,11 @@
       <c r="J45" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>87</v>
       </c>
@@ -2214,8 +2353,11 @@
       <c r="J46" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>88</v>
       </c>
@@ -2246,8 +2388,11 @@
       <c r="J47" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>90</v>
       </c>
@@ -2278,8 +2423,11 @@
       <c r="J48" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>91</v>
       </c>
@@ -2310,8 +2458,11 @@
       <c r="J49" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>92</v>
       </c>
@@ -2342,8 +2493,11 @@
       <c r="J50" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>93</v>
       </c>
@@ -2374,8 +2528,11 @@
       <c r="J51" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>94</v>
       </c>
@@ -2406,8 +2563,11 @@
       <c r="J52" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>95</v>
       </c>
@@ -2438,8 +2598,11 @@
       <c r="J53" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>96</v>
       </c>
@@ -2470,8 +2633,11 @@
       <c r="J54" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>97</v>
       </c>
@@ -2502,8 +2668,11 @@
       <c r="J55" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>98</v>
       </c>
@@ -2534,8 +2703,11 @@
       <c r="J56" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>99</v>
       </c>
@@ -2566,8 +2738,11 @@
       <c r="J57" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>100</v>
       </c>
@@ -2598,8 +2773,11 @@
       <c r="J58" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>101</v>
       </c>
@@ -2630,8 +2808,11 @@
       <c r="J59" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>102</v>
       </c>
@@ -2662,8 +2843,11 @@
       <c r="J60" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>103</v>
       </c>
@@ -2694,8 +2878,11 @@
       <c r="J61" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>104</v>
       </c>
@@ -2726,8 +2913,11 @@
       <c r="J62" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>105</v>
       </c>
@@ -2758,8 +2948,11 @@
       <c r="J63" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>106</v>
       </c>
@@ -2790,8 +2983,11 @@
       <c r="J64" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>75</v>
       </c>
@@ -2822,8 +3018,11 @@
       <c r="J65" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>76</v>
       </c>
@@ -2854,8 +3053,11 @@
       <c r="J66" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>77</v>
       </c>
@@ -2886,8 +3088,11 @@
       <c r="J67" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>78</v>
       </c>
@@ -2918,8 +3123,11 @@
       <c r="J68" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>79</v>
       </c>
@@ -2950,8 +3158,11 @@
       <c r="J69" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>80</v>
       </c>
@@ -2982,8 +3193,11 @@
       <c r="J70" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>81</v>
       </c>
@@ -3014,8 +3228,11 @@
       <c r="J71" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>82</v>
       </c>
@@ -3046,8 +3263,11 @@
       <c r="J72" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>83</v>
       </c>
@@ -3078,8 +3298,11 @@
       <c r="J73" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>84</v>
       </c>
@@ -3110,8 +3333,11 @@
       <c r="J74" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>85</v>
       </c>
@@ -3142,8 +3368,11 @@
       <c r="J75" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>86</v>
       </c>
@@ -3174,8 +3403,11 @@
       <c r="J76" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>87</v>
       </c>
@@ -3206,8 +3438,11 @@
       <c r="J77" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>88</v>
       </c>
@@ -3238,8 +3473,11 @@
       <c r="J78" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>89</v>
       </c>
@@ -3270,8 +3508,11 @@
       <c r="J79" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>90</v>
       </c>
@@ -3302,8 +3543,11 @@
       <c r="J80" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>91</v>
       </c>
@@ -3334,8 +3578,11 @@
       <c r="J81" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>92</v>
       </c>
@@ -3366,8 +3613,11 @@
       <c r="J82" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>93</v>
       </c>
@@ -3398,8 +3648,11 @@
       <c r="J83" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>94</v>
       </c>
@@ -3430,8 +3683,11 @@
       <c r="J84" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>95</v>
       </c>
@@ -3462,8 +3718,11 @@
       <c r="J85" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>96</v>
       </c>
@@ -3494,8 +3753,11 @@
       <c r="J86" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>97</v>
       </c>
@@ -3526,8 +3788,11 @@
       <c r="J87" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>98</v>
       </c>
@@ -3558,8 +3823,11 @@
       <c r="J88" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>99</v>
       </c>
@@ -3590,8 +3858,11 @@
       <c r="J89" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>100</v>
       </c>
@@ -3622,8 +3893,11 @@
       <c r="J90" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>101</v>
       </c>
@@ -3654,8 +3928,11 @@
       <c r="J91" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>102</v>
       </c>
@@ -3686,8 +3963,11 @@
       <c r="J92" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>103</v>
       </c>
@@ -3718,8 +3998,11 @@
       <c r="J93" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>104</v>
       </c>
@@ -3750,8 +4033,11 @@
       <c r="J94" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>105</v>
       </c>
@@ -3782,8 +4068,11 @@
       <c r="J95" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>106</v>
       </c>
@@ -3814,8 +4103,11 @@
       <c r="J96" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>75</v>
       </c>
@@ -3846,8 +4138,11 @@
       <c r="J97" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>76</v>
       </c>
@@ -3878,8 +4173,11 @@
       <c r="J98" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>77</v>
       </c>
@@ -3910,8 +4208,11 @@
       <c r="J99" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>78</v>
       </c>
@@ -3942,8 +4243,11 @@
       <c r="J100" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>79</v>
       </c>
@@ -3974,8 +4278,11 @@
       <c r="J101" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>80</v>
       </c>
@@ -4006,8 +4313,11 @@
       <c r="J102" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>81</v>
       </c>
@@ -4038,8 +4348,11 @@
       <c r="J103" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>82</v>
       </c>
@@ -4070,8 +4383,11 @@
       <c r="J104" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>83</v>
       </c>
@@ -4102,8 +4418,11 @@
       <c r="J105" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>84</v>
       </c>
@@ -4134,8 +4453,11 @@
       <c r="J106" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>85</v>
       </c>
@@ -4166,8 +4488,11 @@
       <c r="J107" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>86</v>
       </c>
@@ -4198,8 +4523,11 @@
       <c r="J108" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K108">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>87</v>
       </c>
@@ -4230,8 +4558,11 @@
       <c r="J109" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>88</v>
       </c>
@@ -4262,8 +4593,11 @@
       <c r="J110" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K110">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>89</v>
       </c>
@@ -4294,8 +4628,11 @@
       <c r="J111" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>90</v>
       </c>
@@ -4326,8 +4663,11 @@
       <c r="J112" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>91</v>
       </c>
@@ -4358,8 +4698,11 @@
       <c r="J113" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K113">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>92</v>
       </c>
@@ -4390,8 +4733,11 @@
       <c r="J114" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>93</v>
       </c>
@@ -4422,8 +4768,11 @@
       <c r="J115" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>94</v>
       </c>
@@ -4454,8 +4803,11 @@
       <c r="J116" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K116">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>95</v>
       </c>
@@ -4486,8 +4838,11 @@
       <c r="J117" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>96</v>
       </c>
@@ -4518,8 +4873,11 @@
       <c r="J118" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K118">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>97</v>
       </c>
@@ -4550,8 +4908,11 @@
       <c r="J119" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>98</v>
       </c>
@@ -4582,8 +4943,11 @@
       <c r="J120" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>99</v>
       </c>
@@ -4614,8 +4978,11 @@
       <c r="J121" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K121">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>100</v>
       </c>
@@ -4646,8 +5013,11 @@
       <c r="J122" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K122">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>101</v>
       </c>
@@ -4678,8 +5048,11 @@
       <c r="J123" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K123">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>102</v>
       </c>
@@ -4710,8 +5083,11 @@
       <c r="J124" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K124">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>103</v>
       </c>
@@ -4742,8 +5118,11 @@
       <c r="J125" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>104</v>
       </c>
@@ -4774,8 +5153,11 @@
       <c r="J126" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>105</v>
       </c>
@@ -4806,8 +5188,11 @@
       <c r="J127" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>106</v>
       </c>
@@ -4838,8 +5223,11 @@
       <c r="J128" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>75</v>
       </c>
@@ -4870,8 +5258,11 @@
       <c r="J129" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>76</v>
       </c>
@@ -4902,8 +5293,11 @@
       <c r="J130" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>77</v>
       </c>
@@ -4934,8 +5328,11 @@
       <c r="J131" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>78</v>
       </c>
@@ -4966,8 +5363,11 @@
       <c r="J132" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>79</v>
       </c>
@@ -4998,8 +5398,11 @@
       <c r="J133" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>80</v>
       </c>
@@ -5030,8 +5433,11 @@
       <c r="J134" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>81</v>
       </c>
@@ -5062,8 +5468,11 @@
       <c r="J135" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>82</v>
       </c>
@@ -5094,8 +5503,11 @@
       <c r="J136" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>83</v>
       </c>
@@ -5126,8 +5538,11 @@
       <c r="J137" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>84</v>
       </c>
@@ -5158,8 +5573,11 @@
       <c r="J138" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>85</v>
       </c>
@@ -5190,8 +5608,11 @@
       <c r="J139" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>86</v>
       </c>
@@ -5222,8 +5643,11 @@
       <c r="J140" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K140">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>87</v>
       </c>
@@ -5254,8 +5678,11 @@
       <c r="J141" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K141">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>88</v>
       </c>
@@ -5286,8 +5713,11 @@
       <c r="J142" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>89</v>
       </c>
@@ -5318,8 +5748,11 @@
       <c r="J143" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>90</v>
       </c>
@@ -5350,8 +5783,11 @@
       <c r="J144" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>91</v>
       </c>
@@ -5382,8 +5818,11 @@
       <c r="J145" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>92</v>
       </c>
@@ -5414,8 +5853,11 @@
       <c r="J146" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>93</v>
       </c>
@@ -5446,8 +5888,11 @@
       <c r="J147" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K147">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>94</v>
       </c>
@@ -5478,8 +5923,11 @@
       <c r="J148" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K148">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>95</v>
       </c>
@@ -5510,8 +5958,11 @@
       <c r="J149" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K149">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>96</v>
       </c>
@@ -5542,8 +5993,11 @@
       <c r="J150" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K150">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>97</v>
       </c>
@@ -5574,8 +6028,11 @@
       <c r="J151" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>98</v>
       </c>
@@ -5606,8 +6063,11 @@
       <c r="J152" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K152">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>99</v>
       </c>
@@ -5638,8 +6098,11 @@
       <c r="J153" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K153">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>100</v>
       </c>
@@ -5670,8 +6133,11 @@
       <c r="J154" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>101</v>
       </c>
@@ -5702,8 +6168,11 @@
       <c r="J155" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>102</v>
       </c>
@@ -5734,8 +6203,11 @@
       <c r="J156" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>103</v>
       </c>
@@ -5766,8 +6238,11 @@
       <c r="J157" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K157">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>104</v>
       </c>
@@ -5798,8 +6273,11 @@
       <c r="J158" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K158">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>105</v>
       </c>
@@ -5830,8 +6308,11 @@
       <c r="J159" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K159">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>106</v>
       </c>
@@ -5862,8 +6343,11 @@
       <c r="J160" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K160">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>75</v>
       </c>
@@ -5894,8 +6378,11 @@
       <c r="J161" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K161">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>76</v>
       </c>
@@ -5926,8 +6413,11 @@
       <c r="J162" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>77</v>
       </c>
@@ -5958,8 +6448,11 @@
       <c r="J163" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K163">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>78</v>
       </c>
@@ -5990,8 +6483,11 @@
       <c r="J164" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K164">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>79</v>
       </c>
@@ -6022,8 +6518,11 @@
       <c r="J165" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K165">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>80</v>
       </c>
@@ -6054,8 +6553,11 @@
       <c r="J166" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K166">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>81</v>
       </c>
@@ -6086,8 +6588,11 @@
       <c r="J167" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K167">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>82</v>
       </c>
@@ -6118,8 +6623,11 @@
       <c r="J168" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K168">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>83</v>
       </c>
@@ -6150,8 +6658,11 @@
       <c r="J169" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K169">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>84</v>
       </c>
@@ -6182,8 +6693,11 @@
       <c r="J170" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K170">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>85</v>
       </c>
@@ -6214,8 +6728,11 @@
       <c r="J171" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K171">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>86</v>
       </c>
@@ -6246,8 +6763,11 @@
       <c r="J172" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K172">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>87</v>
       </c>
@@ -6278,8 +6798,11 @@
       <c r="J173" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K173">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>88</v>
       </c>
@@ -6310,8 +6833,11 @@
       <c r="J174" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K174">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>89</v>
       </c>
@@ -6342,8 +6868,11 @@
       <c r="J175" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K175">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>90</v>
       </c>
@@ -6374,8 +6903,11 @@
       <c r="J176" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K176">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>91</v>
       </c>
@@ -6406,8 +6938,11 @@
       <c r="J177" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K177">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>92</v>
       </c>
@@ -6438,8 +6973,11 @@
       <c r="J178" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K178">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>93</v>
       </c>
@@ -6470,8 +7008,11 @@
       <c r="J179" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K179">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>94</v>
       </c>
@@ -6502,8 +7043,11 @@
       <c r="J180" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K180">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>95</v>
       </c>
@@ -6534,8 +7078,11 @@
       <c r="J181" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K181">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>96</v>
       </c>
@@ -6566,8 +7113,11 @@
       <c r="J182" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K182">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>97</v>
       </c>
@@ -6598,8 +7148,11 @@
       <c r="J183" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K183">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>98</v>
       </c>
@@ -6630,8 +7183,11 @@
       <c r="J184" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K184">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>99</v>
       </c>
@@ -6662,8 +7218,11 @@
       <c r="J185" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K185">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>100</v>
       </c>
@@ -6694,8 +7253,11 @@
       <c r="J186" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K186">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>101</v>
       </c>
@@ -6726,8 +7288,11 @@
       <c r="J187" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K187">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>102</v>
       </c>
@@ -6758,8 +7323,11 @@
       <c r="J188" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K188">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>103</v>
       </c>
@@ -6790,8 +7358,11 @@
       <c r="J189" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K189">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>104</v>
       </c>
@@ -6822,8 +7393,11 @@
       <c r="J190" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K190">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>105</v>
       </c>
@@ -6854,8 +7428,11 @@
       <c r="J191" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K191">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>106</v>
       </c>
@@ -6886,8 +7463,11 @@
       <c r="J192" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K192">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>75</v>
       </c>
@@ -6918,8 +7498,11 @@
       <c r="J193" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K193">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>76</v>
       </c>
@@ -6950,8 +7533,11 @@
       <c r="J194" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K194">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>77</v>
       </c>
@@ -6982,8 +7568,11 @@
       <c r="J195" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K195">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>78</v>
       </c>
@@ -7014,8 +7603,11 @@
       <c r="J196" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K196">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>79</v>
       </c>
@@ -7046,8 +7638,11 @@
       <c r="J197" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K197">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>80</v>
       </c>
@@ -7078,8 +7673,11 @@
       <c r="J198" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K198">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>81</v>
       </c>
@@ -7110,8 +7708,11 @@
       <c r="J199" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K199">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>82</v>
       </c>
@@ -7142,8 +7743,11 @@
       <c r="J200" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K200">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>83</v>
       </c>
@@ -7174,8 +7778,11 @@
       <c r="J201" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="202" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K201">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>84</v>
       </c>
@@ -7206,8 +7813,11 @@
       <c r="J202" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="203" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K202">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>85</v>
       </c>
@@ -7238,8 +7848,11 @@
       <c r="J203" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K203">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>86</v>
       </c>
@@ -7270,8 +7883,11 @@
       <c r="J204" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="205" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K204">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>87</v>
       </c>
@@ -7302,8 +7918,11 @@
       <c r="J205" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="206" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K205">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>88</v>
       </c>
@@ -7334,8 +7953,11 @@
       <c r="J206" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="207" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K206">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>89</v>
       </c>
@@ -7366,8 +7988,11 @@
       <c r="J207" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="208" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K207">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>90</v>
       </c>
@@ -7398,8 +8023,11 @@
       <c r="J208" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K208">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>91</v>
       </c>
@@ -7430,8 +8058,11 @@
       <c r="J209" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K209">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>92</v>
       </c>
@@ -7462,8 +8093,11 @@
       <c r="J210" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K210">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>93</v>
       </c>
@@ -7494,8 +8128,11 @@
       <c r="J211" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K211">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>94</v>
       </c>
@@ -7526,8 +8163,11 @@
       <c r="J212" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K212">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>95</v>
       </c>
@@ -7558,8 +8198,11 @@
       <c r="J213" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K213">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>96</v>
       </c>
@@ -7590,8 +8233,11 @@
       <c r="J214" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K214">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>97</v>
       </c>
@@ -7622,8 +8268,11 @@
       <c r="J215" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>98</v>
       </c>
@@ -7654,8 +8303,11 @@
       <c r="J216" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K216">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>99</v>
       </c>
@@ -7686,8 +8338,11 @@
       <c r="J217" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K217">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>100</v>
       </c>
@@ -7718,8 +8373,11 @@
       <c r="J218" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K218">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>101</v>
       </c>
@@ -7750,8 +8408,11 @@
       <c r="J219" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K219">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>102</v>
       </c>
@@ -7782,8 +8443,11 @@
       <c r="J220" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K220">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>103</v>
       </c>
@@ -7814,8 +8478,11 @@
       <c r="J221" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K221">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>104</v>
       </c>
@@ -7846,8 +8513,11 @@
       <c r="J222" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K222">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>105</v>
       </c>
@@ -7878,8 +8548,11 @@
       <c r="J223" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K223">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>106</v>
       </c>
@@ -7908,6 +8581,9 @@
         <v>0</v>
       </c>
       <c r="J224" s="1">
+        <v>0</v>
+      </c>
+      <c r="K224">
         <v>0</v>
       </c>
     </row>

</xml_diff>